<commit_message>
Fill in unit costs for the new Topology A BOM parts
Q4-Q7 PMXB43UNEZ (C547273) at $0.5441 and R53-R56 1K (C11702) at
$0.0013, both LCSC 100+ pricing. Re-checked every designator, value and
footprint against the current schematic and PCB: all 118 placed parts
are accounted for, with no extra or missing rows.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/RocketLocatorBOM.xlsx
+++ b/BOM/RocketLocatorBOM.xlsx
@@ -2765,9 +2765,12 @@
           <t xml:space="preserve">Extended</t>
         </is>
       </c>
+      <c r="H23">
+        <v>0.5441</v>
+      </c>
       <c r="I23" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
+        <v>2.1764</v>
       </c>
       <c r="K23">
         <v>4</v>
@@ -2782,7 +2785,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t xml:space="preserve">New: deploy low-side FETs (Topology A); unit cost not yet looked up</t>
+          <t xml:space="preserve">New: deploy low-side FETs (Topology A); PMXB43UNEZ, unit cost is LCSC 100+ price (Oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3599,9 +3602,12 @@
           <t xml:space="preserve">Basic</t>
         </is>
       </c>
+      <c r="H41">
+        <v>0.0013</v>
+      </c>
       <c r="I41" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
+        <v>0.0052</v>
       </c>
       <c r="K41">
         <v>10</v>
@@ -3616,7 +3622,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t xml:space="preserve">New: DEPLOY1+..4+ bleeders (Topology A); unit cost not yet looked up</t>
+          <t xml:space="preserve">New: DEPLOY1+..4+ bleeders (Topology A); unit cost is LCSC 100+ price (Oct 2026)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price the BOM from JLCPCB
Unit Cost and Type for every orderable row now come from JLCPCB's parts
API (2026-10-21), using the price tier that matches each row's Quantity
Needed. Assumptions sheet records the source and date. Notes flag C7
(C2981728) out of stock at JLCPCB with a 30-piece gap, C26 now Basic,
and the D4/D5 part (C22461785) being XL-Z1921RGBA-SG while KiCad says
XL-Z1912RGBA-SG.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qn4Fhe37cECFfk8PPTy8Kj
</commit_message>
<xml_diff>
--- a/BOM/RocketLocatorBOM.xlsx
+++ b/BOM/RocketLocatorBOM.xlsx
@@ -1901,15 +1901,17 @@
       <c r="F2" t="s">
         <v>114</v>
       </c>
-      <c r="G2" t="s">
-        <v>115</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H2">
-        <v>1.21E-2</v>
+        <v>0.022</v>
       </c>
       <c r="I2" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0363</v>
+        <v>0.066</v>
       </c>
       <c r="J2">
         <v>210</v>
@@ -1948,15 +1950,17 @@
       <c r="F3" t="s">
         <v>118</v>
       </c>
-      <c r="G3" t="s">
-        <v>117</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H3">
-        <v>1.4E-3</v>
+        <v>0.0041</v>
       </c>
       <c r="I3" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0014</v>
+        <v>0.0041</v>
       </c>
       <c r="J3">
         <v>60</v>
@@ -1995,15 +1999,17 @@
       <c r="F4" t="s">
         <v>116</v>
       </c>
-      <c r="G4" t="s">
-        <v>117</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H4">
-        <v>3.3999999999999998E-3</v>
+        <v>0.0257</v>
       </c>
       <c r="I4" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0034</v>
+        <v>0.0257</v>
       </c>
       <c r="J4">
         <v>930</v>
@@ -2042,15 +2048,17 @@
       <c r="F5" t="s">
         <v>119</v>
       </c>
-      <c r="G5" t="s">
-        <v>117</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H5">
-        <v>3.3E-3</v>
+        <v>0.0075</v>
       </c>
       <c r="I5" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0297</v>
+        <v>0.0675</v>
       </c>
       <c r="J5">
         <v>480</v>
@@ -2089,15 +2097,17 @@
       <c r="F6" t="s">
         <v>120</v>
       </c>
-      <c r="G6" t="s">
-        <v>117</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H6">
-        <v>1.2999999999999999E-3</v>
+        <v>0.0055</v>
       </c>
       <c r="I6" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0091</v>
+        <v>0.0385</v>
       </c>
       <c r="J6">
         <v>300</v>
@@ -2136,15 +2146,17 @@
       <c r="F7" t="s">
         <v>171</v>
       </c>
-      <c r="G7" t="s">
-        <v>115</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H7">
-        <v>0.35070000000000001</v>
+        <v>0.5363</v>
       </c>
       <c r="I7" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.3507</v>
+        <v>0.5363</v>
       </c>
       <c r="L7">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
@@ -2154,8 +2166,10 @@
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v>30</v>
       </c>
-      <c r="Q7" t="s">
-        <v>179</v>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C0G; JLCPCB stock 0 &lt; gap 30 (2026-10-21)</t>
+        </is>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.45">
@@ -2177,15 +2191,17 @@
       <c r="F8" t="s">
         <v>178</v>
       </c>
-      <c r="G8" t="s">
-        <v>115</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H8">
-        <v>7.0999999999999994E-2</v>
+        <v>0.168</v>
       </c>
       <c r="I8" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.071</v>
+        <v>0.168</v>
       </c>
       <c r="J8">
         <v>150</v>
@@ -2201,8 +2217,10 @@
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-      <c r="Q8" t="s">
-        <v>168</v>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X5R; JLCPCB now lists as Basic (was Extended)</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.45">
@@ -2224,15 +2242,17 @@
       <c r="F9" t="s">
         <v>177</v>
       </c>
-      <c r="G9" t="s">
-        <v>115</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H9">
-        <v>4.7000000000000002E-3</v>
+        <v>0.0157</v>
       </c>
       <c r="I9" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0047</v>
+        <v>0.0157</v>
       </c>
       <c r="J9">
         <v>500</v>
@@ -2268,15 +2288,17 @@
       <c r="F10" t="s">
         <v>121</v>
       </c>
-      <c r="G10" t="s">
-        <v>115</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H10">
-        <v>8.8000000000000005E-3</v>
+        <v>0.013</v>
       </c>
       <c r="I10" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0088</v>
+        <v>0.013</v>
       </c>
       <c r="J10">
         <v>400</v>
@@ -2293,7 +2315,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2312,15 +2334,17 @@
       <c r="F11" t="s">
         <v>122</v>
       </c>
-      <c r="G11" t="s">
-        <v>115</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H11">
-        <v>1.5900000000000001E-2</v>
+        <v>0.0158</v>
       </c>
       <c r="I11" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0318</v>
+        <v>0.0316</v>
       </c>
       <c r="J11">
         <v>72</v>
@@ -2335,6 +2359,11 @@
       <c r="M11" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JLCPCB part is XL-Z1921RGBA-SG; KiCad value/footprint say XL-Z1912RGBA-SG</t>
+        </is>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.45">
@@ -2388,15 +2417,17 @@
       <c r="F13" t="s">
         <v>124</v>
       </c>
-      <c r="G13" t="s">
-        <v>115</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H13">
-        <v>3.32E-2</v>
+        <v>0.0635</v>
       </c>
       <c r="I13" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0332</v>
+        <v>0.0635</v>
       </c>
       <c r="J13">
         <v>257</v>
@@ -2559,15 +2590,17 @@
       <c r="F18" t="s">
         <v>125</v>
       </c>
-      <c r="G18" t="s">
-        <v>115</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H18">
-        <v>2.4799999999999999E-2</v>
+        <v>0.0417</v>
       </c>
       <c r="I18" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0248</v>
+        <v>0.0417</v>
       </c>
       <c r="J18">
         <v>279</v>
@@ -2664,15 +2697,17 @@
       <c r="F21" t="s">
         <v>126</v>
       </c>
-      <c r="G21" t="s">
-        <v>115</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H21">
-        <v>2.0899999999999998E-2</v>
+        <v>0.0218</v>
       </c>
       <c r="I21" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0209</v>
+        <v>0.0218</v>
       </c>
       <c r="J21">
         <v>75</v>
@@ -2708,15 +2743,17 @@
       <c r="F22" t="s">
         <v>127</v>
       </c>
-      <c r="G22" t="s">
-        <v>115</v>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H22">
-        <v>3.9199999999999999E-2</v>
+        <v>0.0403</v>
       </c>
       <c r="I22" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0392</v>
+        <v>0.0403</v>
       </c>
       <c r="J22">
         <v>42</v>
@@ -2762,15 +2799,15 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Extended</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H23">
-        <v>0.5441</v>
+        <v>0.5428</v>
       </c>
       <c r="I23" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>2.1764</v>
+        <v>2.1712</v>
       </c>
       <c r="K23">
         <v>4</v>
@@ -2808,15 +2845,17 @@
       <c r="F24" t="s">
         <v>128</v>
       </c>
-      <c r="G24" t="s">
-        <v>115</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H24">
-        <v>2.9999999999999997E-4</v>
+        <v>0.0014</v>
       </c>
       <c r="I24" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0006</v>
+        <v>0.0028</v>
       </c>
       <c r="J24">
         <v>2930</v>
@@ -2854,15 +2893,17 @@
           <t xml:space="preserve">C25207446</t>
         </is>
       </c>
-      <c r="G25" t="s">
-        <v>115</v>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H25">
-        <v>2.0500000000000001E-2</v>
+        <v>0.0203</v>
       </c>
       <c r="I25" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0205</v>
+        <v>0.0203</v>
       </c>
       <c r="J25">
         <v>100</v>
@@ -2898,15 +2939,17 @@
       <c r="F26" t="s">
         <v>129</v>
       </c>
-      <c r="G26" t="s">
-        <v>117</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H26">
-        <v>8.0000000000000004E-4</v>
+        <v>0.0011</v>
       </c>
       <c r="I26" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0008</v>
+        <v>0.0011</v>
       </c>
       <c r="J26">
         <v>80</v>
@@ -2947,15 +2990,17 @@
       <c r="F27" t="s">
         <v>131</v>
       </c>
-      <c r="G27" t="s">
-        <v>115</v>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H27">
-        <v>8.0000000000000004E-4</v>
+        <v>0.0019</v>
       </c>
       <c r="I27" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.004</v>
+        <v>0.0095</v>
       </c>
       <c r="J27">
         <v>150</v>
@@ -2993,15 +3038,17 @@
       <c r="F28" t="s">
         <v>132</v>
       </c>
-      <c r="G28" t="s">
-        <v>117</v>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H28">
-        <v>8.0000000000000004E-4</v>
+        <v>0.0015</v>
       </c>
       <c r="I28" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0024</v>
+        <v>0.0045</v>
       </c>
       <c r="J28">
         <v>150</v>
@@ -3037,15 +3084,17 @@
       <c r="F29" t="s">
         <v>133</v>
       </c>
-      <c r="G29" t="s">
-        <v>117</v>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H29">
-        <v>8.0000000000000004E-4</v>
+        <v>0.0012</v>
       </c>
       <c r="I29" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0008</v>
+        <v>0.0012</v>
       </c>
       <c r="J29">
         <v>74</v>
@@ -3081,15 +3130,17 @@
       <c r="F30" t="s">
         <v>134</v>
       </c>
-      <c r="G30" t="s">
-        <v>117</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H30">
-        <v>4.0000000000000002E-4</v>
+        <v>0.0034</v>
       </c>
       <c r="I30" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0008</v>
+        <v>0.0068</v>
       </c>
       <c r="J30">
         <v>890</v>
@@ -3125,15 +3176,17 @@
       <c r="F31" t="s">
         <v>135</v>
       </c>
-      <c r="G31" t="s">
-        <v>117</v>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H31">
-        <v>8.0000000000000004E-4</v>
+        <v>0.002</v>
       </c>
       <c r="I31" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0032</v>
+        <v>0.008</v>
       </c>
       <c r="J31">
         <v>150</v>
@@ -3169,15 +3222,17 @@
       <c r="F32" t="s">
         <v>136</v>
       </c>
-      <c r="G32" t="s">
-        <v>115</v>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H32">
-        <v>1E-4</v>
+        <v>0.0026</v>
       </c>
       <c r="I32" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0007</v>
+        <v>0.0182</v>
       </c>
       <c r="J32">
         <v>9705</v>
@@ -3213,15 +3268,17 @@
       <c r="F33" t="s">
         <v>162</v>
       </c>
-      <c r="G33" t="s">
-        <v>117</v>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H33">
-        <v>4.0000000000000002E-4</v>
+        <v>0.0021</v>
       </c>
       <c r="I33" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0008</v>
+        <v>0.0042</v>
       </c>
       <c r="J33">
         <v>970</v>
@@ -3259,15 +3316,17 @@
       <c r="F34" t="s">
         <v>130</v>
       </c>
-      <c r="G34" t="s">
-        <v>117</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H34">
-        <v>4.0000000000000002E-4</v>
+        <v>0.0012</v>
       </c>
       <c r="I34" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0036</v>
+        <v>0.0108</v>
       </c>
       <c r="J34">
         <v>960</v>
@@ -3308,15 +3367,17 @@
       <c r="F35" t="s">
         <v>137</v>
       </c>
-      <c r="G35" t="s">
-        <v>115</v>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H35">
-        <v>2.9999999999999997E-4</v>
+        <v>0.0012</v>
       </c>
       <c r="I35" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0009</v>
+        <v>0.0036</v>
       </c>
       <c r="J35">
         <v>2940</v>
@@ -3352,15 +3413,17 @@
       <c r="F36" t="s">
         <v>138</v>
       </c>
-      <c r="G36" t="s">
-        <v>117</v>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H36">
-        <v>8.0000000000000004E-4</v>
+        <v>0.0018</v>
       </c>
       <c r="I36" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0008</v>
+        <v>0.0018</v>
       </c>
       <c r="J36">
         <v>3030</v>
@@ -3401,11 +3464,13 @@
       <c r="F37" t="s">
         <v>139</v>
       </c>
-      <c r="G37" t="s">
-        <v>115</v>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H37">
-        <v>5.9999999999999995E-4</v>
+        <v>0.0006</v>
       </c>
       <c r="I37" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
@@ -3450,15 +3515,17 @@
       <c r="F38" t="s">
         <v>140</v>
       </c>
-      <c r="G38" t="s">
-        <v>115</v>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H38">
-        <v>6.9999999999999999E-4</v>
+        <v>0.0023</v>
       </c>
       <c r="I38" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0007</v>
+        <v>0.0023</v>
       </c>
       <c r="J38">
         <v>60</v>
@@ -3494,15 +3561,17 @@
       <c r="F39" t="s">
         <v>173</v>
       </c>
-      <c r="G39" t="s">
-        <v>115</v>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H39">
-        <v>2.0500000000000001E-2</v>
+        <v>0.0213</v>
       </c>
       <c r="I39" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0205</v>
+        <v>0.0213</v>
       </c>
       <c r="J39">
         <v>100</v>
@@ -3540,15 +3609,17 @@
       <c r="F40" t="s">
         <v>141</v>
       </c>
-      <c r="G40" t="s">
-        <v>117</v>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
       </c>
       <c r="H40">
-        <v>5.0000000000000001E-4</v>
+        <v>0.0015</v>
       </c>
       <c r="I40" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.004</v>
+        <v>0.012</v>
       </c>
       <c r="J40">
         <v>4960</v>
@@ -3599,7 +3670,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Basic</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H41">
@@ -3645,15 +3716,17 @@
       <c r="F42" t="s">
         <v>142</v>
       </c>
-      <c r="G42" t="s">
-        <v>115</v>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H42">
-        <v>0.45190000000000002</v>
+        <v>0.5919</v>
       </c>
       <c r="I42" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>2.2595</v>
+        <v>2.9595</v>
       </c>
       <c r="J42">
         <v>120</v>
@@ -3689,15 +3762,17 @@
       <c r="F43" t="s">
         <v>143</v>
       </c>
-      <c r="G43" t="s">
-        <v>115</v>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H43">
-        <v>0.3508</v>
+        <v>0.3336</v>
       </c>
       <c r="I43" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.3508</v>
+        <v>0.3336</v>
       </c>
       <c r="J43">
         <v>30</v>
@@ -3735,15 +3810,17 @@
       <c r="F44" t="s">
         <v>155</v>
       </c>
-      <c r="G44" t="s">
-        <v>115</v>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H44">
-        <v>0.3856</v>
+        <v>0.3679</v>
       </c>
       <c r="I44" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.3856</v>
+        <v>0.3679</v>
       </c>
       <c r="J44">
         <v>50</v>
@@ -3782,15 +3859,17 @@
       <c r="F45" t="s">
         <v>144</v>
       </c>
-      <c r="G45" t="s">
-        <v>115</v>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H45">
-        <v>0.2535</v>
+        <v>0.7504</v>
       </c>
       <c r="I45" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.2535</v>
+        <v>0.7504</v>
       </c>
       <c r="J45">
         <v>0</v>
@@ -3829,15 +3908,17 @@
       <c r="F46" t="s">
         <v>145</v>
       </c>
-      <c r="G46" t="s">
-        <v>115</v>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H46">
-        <v>8.0976999999999997</v>
+        <v>14.1006</v>
       </c>
       <c r="I46" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>8.0977</v>
+        <v>14.1006</v>
       </c>
       <c r="J46">
         <v>30</v>
@@ -3873,15 +3954,17 @@
       <c r="F47" t="s">
         <v>146</v>
       </c>
-      <c r="G47" t="s">
-        <v>115</v>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H47">
-        <v>5.2519999999999998</v>
+        <v>5.467</v>
       </c>
       <c r="I47" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>5.252</v>
+        <v>5.467</v>
       </c>
       <c r="J47">
         <v>30</v>
@@ -3917,15 +4000,17 @@
       <c r="F48" t="s">
         <v>147</v>
       </c>
-      <c r="G48" t="s">
-        <v>115</v>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H48">
-        <v>0.92589999999999995</v>
+        <v>2.0322</v>
       </c>
       <c r="I48" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.9259</v>
+        <v>2.0322</v>
       </c>
       <c r="J48">
         <v>30</v>
@@ -3961,15 +4046,17 @@
       <c r="F49" t="s">
         <v>148</v>
       </c>
-      <c r="G49" t="s">
-        <v>115</v>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H49">
-        <v>1.2314000000000001</v>
+        <v>1.1346</v>
       </c>
       <c r="I49" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>1.2314</v>
+        <v>1.1346</v>
       </c>
       <c r="J49">
         <v>0</v>
@@ -4008,15 +4095,17 @@
       <c r="F50" t="s">
         <v>149</v>
       </c>
-      <c r="G50" t="s">
-        <v>115</v>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H50">
-        <v>24.545999999999999</v>
+        <v>20.5582</v>
       </c>
       <c r="I50" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>24.546</v>
+        <v>20.5582</v>
       </c>
       <c r="J50">
         <v>30</v>
@@ -4052,15 +4141,17 @@
       <c r="F51" t="s">
         <v>150</v>
       </c>
-      <c r="G51" t="s">
-        <v>115</v>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H51">
-        <v>0.17349999999999999</v>
+        <v>0.2927</v>
       </c>
       <c r="I51" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.1735</v>
+        <v>0.2927</v>
       </c>
       <c r="J51">
         <v>60</v>
@@ -4096,15 +4187,17 @@
       <c r="F52" t="s">
         <v>152</v>
       </c>
-      <c r="G52" t="s">
-        <v>115</v>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H52">
-        <v>0.41399999999999998</v>
+        <v>0.4284</v>
       </c>
       <c r="I52" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.414</v>
+        <v>0.4284</v>
       </c>
       <c r="J52">
         <v>30</v>
@@ -4140,15 +4233,17 @@
       <c r="F53" t="s">
         <v>151</v>
       </c>
-      <c r="G53" t="s">
-        <v>115</v>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H53">
-        <v>20.32</v>
+        <v>24.6878</v>
       </c>
       <c r="I53" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>20.32</v>
+        <v>24.6878</v>
       </c>
       <c r="J53">
         <v>30</v>
@@ -4184,15 +4279,17 @@
       <c r="F54" t="s">
         <v>153</v>
       </c>
-      <c r="G54" t="s">
-        <v>115</v>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
       </c>
       <c r="H54">
-        <v>6.3399999999999998E-2</v>
+        <v>0.1196</v>
       </c>
       <c r="I54" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0634</v>
+        <v>0.1196</v>
       </c>
       <c r="J54">
         <v>127</v>
@@ -4222,7 +4319,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="26" style="2" customWidth="1"/>
@@ -4236,6 +4333,18 @@
       </c>
       <c r="B1" s="2">
         <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Unit cost source</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>JLCPCB parts API, 2026-10-21; price tier for each row's Quantity Needed (USD)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move C7 (BATTLVL filter) to 0402 X7R
C7 only filters the battery-sense divider node (max ~3.2 V), so the
out-of-stock 50 V C0G 1206 part is not needed. Swap it to the same
0.1uF 0402 X7R as the other decoupling caps (C1525):
- Schematic footprint Capacitor_SMD:C_0402_1005Metric
- PCB: 0402 placed vertically on B.Cu at (41.775, 30.16) on the
  existing BATTLVL node; GND pad picks up the B.Cu pour. Old GND stub
  removed, zones refilled. DRC: 0 errors, 0 unconnected, schematic
  parity clean.
- BOM: C7 merged into the 0.1uF row, its own row removed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qn4Fhe37cECFfk8PPTy8Kj
</commit_message>
<xml_diff>
--- a/BOM/RocketLocatorBOM.xlsx
+++ b/BOM/RocketLocatorBOM.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Assumptions" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="1" hidden="1">'RocketLocator'!$A$1:$E$54</definedName>
+    <definedName name="ExternalData_1" localSheetId="1" hidden="1">'RocketLocator'!$A$1:$E$53</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -756,10 +756,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}" name="RocketLocator" displayName="RocketLocator" ref="A1:Q54" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:Q54" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P54">
-    <sortCondition ref="B2:B54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}" name="RocketLocator" displayName="RocketLocator" ref="A1:Q53" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:Q53" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P53">
+    <sortCondition ref="B2:B53"/>
   </sortState>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{0660759B-7B44-48B6-BB59-01895697A8CF}" uniqueName="1" name="Id" queryTableFieldId="1"/>
@@ -1107,7 +1107,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61E55C0D-EF73-420E-9FF2-D4B1756536CB}">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.3984375" bestFit="1" customWidth="1"/>
@@ -1190,8 +1190,10 @@
       <c r="A6" t="s">
         <v>27</v>
       </c>
-      <c r="B6" t="s">
-        <v>192</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>C1,C6,C7,C8,C9,C10,C20,C36</t>
+        </is>
       </c>
       <c r="C6" t="s">
         <v>15</v>
@@ -1202,603 +1204,589 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>159</v>
       </c>
       <c r="B7" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C7" t="s">
         <v>172</v>
       </c>
       <c r="D7" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B8" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="C8" t="s">
-        <v>172</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>166</v>
+        <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>158</v>
+        <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>67</v>
       </c>
       <c r="D9" t="s">
-        <v>177</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
+        <v>39</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HRS_U.FL-R-SMT(01)</t>
+        </is>
       </c>
       <c r="D12" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HRS_U.FL-R-SMT(01)</t>
-        </is>
+        <v>163</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>163</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
         <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" t="s">
-        <v>127</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PMXB43UNE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q4,Q5,Q6,Q7</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nexperia_DFN1010D-3_SOT1215</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C547273</t>
+        </is>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PMXB43UNE</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Q4,Q5,Q6,Q7</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nexperia_DFN1010D-3_SOT1215</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C547273</t>
-        </is>
+      <c r="A16" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>87</v>
+        <v>175</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="C17" t="s">
         <v>7</v>
       </c>
-      <c r="D17" t="s">
-        <v>128</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C25207446</t>
+        </is>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>175</v>
+      <c r="A18">
+        <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="C18" t="s">
         <v>7</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C25207446</t>
-        </is>
+      <c r="D18" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A19">
-        <v>33</v>
+      <c r="A19" t="s">
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>183</v>
       </c>
       <c r="C19" t="s">
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" t="s">
-        <v>183</v>
+        <v>21</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R3,R17,R30</t>
+        </is>
       </c>
       <c r="C20" t="s">
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R3,R17,R30</t>
-        </is>
+        <v>97</v>
+      </c>
+      <c r="B21" t="s">
+        <v>96</v>
       </c>
       <c r="C21" t="s">
         <v>7</v>
       </c>
       <c r="D21" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>97</v>
+        <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>96</v>
+        <v>185</v>
       </c>
       <c r="C22" t="s">
         <v>7</v>
       </c>
       <c r="D22" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="B23" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C23" t="s">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="B24" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C24" t="s">
         <v>7</v>
       </c>
       <c r="D24" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>20</v>
+        <v>161</v>
       </c>
       <c r="B25" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="C25" t="s">
         <v>7</v>
       </c>
       <c r="D25" t="s">
-        <v>136</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>161</v>
-      </c>
-      <c r="B26" t="s">
-        <v>160</v>
+        <v>11</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R4,R16,R19,R35,R43,R45,R46,R47,R48</t>
+        </is>
       </c>
       <c r="C26" t="s">
         <v>7</v>
       </c>
       <c r="D26" t="s">
-        <v>162</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R4,R16,R19,R35,R43,R45,R46,R47,R48</t>
-        </is>
+        <v>29</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
       </c>
       <c r="C27" t="s">
         <v>7</v>
       </c>
       <c r="D27" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
-        <v>29</v>
+      <c r="A28">
+        <v>220</v>
       </c>
       <c r="B28" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C28" t="s">
         <v>7</v>
       </c>
       <c r="D28" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29">
-        <v>220</v>
+        <v>374</v>
       </c>
       <c r="B29" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="C29" t="s">
         <v>7</v>
       </c>
       <c r="D29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A30">
-        <v>374</v>
+      <c r="A30" t="s">
+        <v>99</v>
       </c>
       <c r="B30" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="C30" t="s">
         <v>7</v>
       </c>
       <c r="D30" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>99</v>
+        <v>176</v>
       </c>
       <c r="B31" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="C31" t="s">
         <v>7</v>
       </c>
       <c r="D31" t="s">
-        <v>140</v>
+        <v>173</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>176</v>
-      </c>
-      <c r="B32" t="s">
-        <v>77</v>
+        <v>164</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R20,R29,R42,R44,R49,R50,R51,R52</t>
+        </is>
       </c>
       <c r="C32" t="s">
         <v>7</v>
       </c>
       <c r="D32" t="s">
-        <v>173</v>
+        <v>141</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
-        <v>164</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1K</t>
+        </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">R20,R29,R42,R44,R49,R50,R51,R52</t>
-        </is>
-      </c>
-      <c r="C33" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33" t="s">
-        <v>141</v>
+          <t xml:space="preserve">R53,R54,R55,R56</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R_0402_1005Metric</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C11702</t>
+        </is>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1K</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R53,R54,R55,R56</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R_0402_1005Metric</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C11702</t>
-        </is>
+      <c r="A34" t="s">
+        <v>14</v>
+      </c>
+      <c r="B34" t="s">
+        <v>190</v>
+      </c>
+      <c r="C34" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="B35" t="s">
-        <v>190</v>
+        <v>93</v>
       </c>
       <c r="C35" t="s">
-        <v>13</v>
+        <v>94</v>
       </c>
       <c r="D35" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>95</v>
+        <v>156</v>
       </c>
       <c r="B36" t="s">
-        <v>93</v>
-      </c>
-      <c r="C36" t="s">
-        <v>94</v>
+        <v>100</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WQFN 14 3.00 mm × 2.50 mm</t>
+        </is>
       </c>
       <c r="D36" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>156</v>
+        <v>80</v>
       </c>
       <c r="B37" t="s">
-        <v>100</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WQFN 14 3.00 mm × 2.50 mm</t>
-        </is>
+        <v>78</v>
+      </c>
+      <c r="C37" t="s">
+        <v>79</v>
       </c>
       <c r="D37" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
+        <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>79</v>
+        <v>5</v>
       </c>
       <c r="D38" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>6</v>
+        <v>59</v>
       </c>
       <c r="B39" t="s">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="C39" t="s">
-        <v>5</v>
+        <v>58</v>
       </c>
       <c r="D39" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="B40" t="s">
-        <v>57</v>
+        <v>90</v>
       </c>
       <c r="C40" t="s">
-        <v>58</v>
+        <v>91</v>
       </c>
       <c r="D40" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="B41" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="C41" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="D41" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>82</v>
+        <v>48</v>
       </c>
       <c r="B42" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="C42" t="s">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="D42" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="B43" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="C43" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="D43" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="B44" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="C44" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D44" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="B45" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="C45" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="D45" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B46" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="C46" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="D46" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A47" t="s">
-        <v>74</v>
-      </c>
-      <c r="B47" t="s">
-        <v>72</v>
-      </c>
-      <c r="C47" t="s">
-        <v>73</v>
-      </c>
-      <c r="D47" t="s">
         <v>153</v>
       </c>
     </row>
@@ -1809,7 +1797,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E42B2C4-1B89-42AA-B989-7F67271C8485}">
-  <dimension ref="A1:Q54"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="4.46484375" bestFit="1" customWidth="1"/>
@@ -2082,14 +2070,16 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>192</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>C1,C6,C7,C8,C9,C10,C20,C36</t>
+        </is>
       </c>
       <c r="C6" t="s">
         <v>15</v>
       </c>
       <c r="D6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" t="s">
         <v>27</v>
@@ -2132,7 +2122,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C7" t="s">
         <v>172</v>
@@ -2141,34 +2131,40 @@
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>159</v>
       </c>
       <c r="F7" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H7">
-        <v>0.5363</v>
+        <v>0.168</v>
       </c>
       <c r="I7" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.5363</v>
+        <v>0.168</v>
+      </c>
+      <c r="J7">
+        <v>150</v>
+      </c>
+      <c r="K7">
+        <v>4</v>
       </c>
       <c r="L7">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>30</v>
-      </c>
-      <c r="M7">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>30</v>
+        <v>34</v>
+      </c>
+      <c r="M7" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t xml:space="preserve">C0G; JLCPCB stock 0 &lt; gap 30 (2026-10-21)</t>
+          <t xml:space="preserve">X5R; JLCPCB now lists as Basic (was Extended)</t>
         </is>
       </c>
     </row>
@@ -2177,70 +2173,65 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="C8" t="s">
-        <v>172</v>
+        <v>15</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="F8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H8">
-        <v>0.168</v>
+        <v>0.0157</v>
       </c>
       <c r="I8" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.168</v>
+        <v>0.0157</v>
       </c>
       <c r="J8">
-        <v>150</v>
-      </c>
-      <c r="K8">
-        <v>4</v>
+        <v>500</v>
       </c>
       <c r="L8">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="M8" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X5R; JLCPCB now lists as Basic (was Extended)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="Q8" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>158</v>
+        <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>67</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>166</v>
+        <v>68</v>
       </c>
       <c r="F9" t="s">
-        <v>177</v>
+        <v>121</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2248,45 +2239,45 @@
         </is>
       </c>
       <c r="H9">
-        <v>0.0157</v>
+        <v>0.013</v>
       </c>
       <c r="I9" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0157</v>
+        <v>0.013</v>
       </c>
       <c r="J9">
-        <v>500</v>
+        <v>400</v>
+      </c>
+      <c r="K9">
+        <v>10</v>
       </c>
       <c r="L9">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="M9" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-      <c r="Q9" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="F10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2294,76 +2285,62 @@
         </is>
       </c>
       <c r="H10">
-        <v>0.013</v>
+        <v>0.0158</v>
       </c>
       <c r="I10" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.013</v>
+        <v>0.0316</v>
       </c>
       <c r="J10">
-        <v>400</v>
+        <v>72</v>
       </c>
       <c r="K10">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L10">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="M10" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JLCPCB part is XL-Z1921RGBA-SG; KiCad value/footprint say XL-Z1912RGBA-SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>181</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E11" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="F11" t="s">
-        <v>122</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="H11">
-        <v>0.0158</v>
+        <v>123</v>
       </c>
       <c r="I11" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0316</v>
-      </c>
-      <c r="J11">
-        <v>72</v>
-      </c>
-      <c r="K11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L11">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="M11" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">JLCPCB part is XL-Z1921RGBA-SG; KiCad value/footprint say XL-Z1912RGBA-SG</t>
-        </is>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.45">
@@ -2371,27 +2348,38 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>181</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F12" t="s">
-        <v>123</v>
+        <v>124</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="H12">
+        <v>0.0635</v>
       </c>
       <c r="I12" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
+        <v>0.0635</v>
+      </c>
+      <c r="J12">
+        <v>257</v>
       </c>
       <c r="L12">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="M12" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -2403,38 +2391,27 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
       <c r="E13" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="F13" t="s">
-        <v>124</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="H13">
-        <v>0.0635</v>
+        <v>123</v>
       </c>
       <c r="I13" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0635</v>
-      </c>
-      <c r="J13">
-        <v>257</v>
+        <v>0</v>
       </c>
       <c r="L13">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="M13" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -2446,7 +2423,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
         <v>31</v>
@@ -2455,7 +2432,7 @@
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="F14" t="s">
         <v>123</v>
@@ -2478,16 +2455,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C15" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="F15" t="s">
         <v>123</v>
@@ -2510,16 +2487,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="C16" t="s">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="F16" t="s">
         <v>123</v>
@@ -2542,27 +2519,40 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" t="s">
-        <v>31</v>
+        <v>39</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HRS_U.FL-R-SMT(01)</t>
+        </is>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="F17" t="s">
-        <v>123</v>
+        <v>125</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="H17">
+        <v>0.0417</v>
       </c>
       <c r="I17" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
+        <v>0.0417</v>
+      </c>
+      <c r="J17">
+        <v>279</v>
       </c>
       <c r="L17">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="M17" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -2574,40 +2564,27 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HRS_U.FL-R-SMT(01)</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="C18" t="s">
+        <v>25</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="F18" t="s">
-        <v>125</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="H18">
-        <v>0.0417</v>
+        <v>123</v>
       </c>
       <c r="I18" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0417</v>
-      </c>
-      <c r="J18">
-        <v>279</v>
+        <v>0</v>
       </c>
       <c r="L18">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="M18" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -2619,16 +2596,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="C19" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="D19">
         <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="F19" t="s">
         <v>123</v>
@@ -2651,27 +2628,41 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>53</v>
+        <v>163</v>
       </c>
       <c r="C20" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="D20">
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="F20" t="s">
-        <v>123</v>
+        <v>126</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="H20">
+        <v>0.0218</v>
       </c>
       <c r="I20" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
+        <v>0.0218</v>
+      </c>
+      <c r="J20">
+        <v>75</v>
+      </c>
+      <c r="K20">
+        <v>5</v>
       </c>
       <c r="L20">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="M20" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -2683,7 +2674,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>163</v>
+        <v>17</v>
       </c>
       <c r="C21" t="s">
         <v>18</v>
@@ -2692,10 +2683,10 @@
         <v>1</v>
       </c>
       <c r="E21" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F21" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -2703,45 +2694,53 @@
         </is>
       </c>
       <c r="H21">
-        <v>0.0218</v>
+        <v>0.0403</v>
       </c>
       <c r="I21" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0218</v>
+        <v>0.0403</v>
       </c>
       <c r="J21">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="K21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L21">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M21" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" t="s">
-        <v>18</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q4,Q5,Q6,Q7</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nexperia_DFN1010D-3_SOT1215</t>
+        </is>
       </c>
       <c r="D22">
-        <v>1</v>
-      </c>
-      <c r="E22" t="s">
-        <v>19</v>
-      </c>
-      <c r="F22" t="s">
-        <v>127</v>
+        <v>4</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PMXB43UNE</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C547273</t>
+        </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -2749,53 +2748,47 @@
         </is>
       </c>
       <c r="H22">
-        <v>0.0403</v>
+        <v>0.5428</v>
       </c>
       <c r="I22" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0403</v>
-      </c>
-      <c r="J22">
-        <v>42</v>
+        <v>2.1712</v>
       </c>
       <c r="K22">
         <v>4</v>
       </c>
       <c r="L22">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>34</v>
-      </c>
-      <c r="M22" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.45">
+        <v>124</v>
+      </c>
+      <c r="M22">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v>124</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New: deploy low-side FETs (Topology A); PMXB43UNEZ, unit cost is LCSC 100+ price (Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Q4,Q5,Q6,Q7</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nexperia_DFN1010D-3_SOT1215</t>
-        </is>
+      <c r="B23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C23" t="s">
+        <v>7</v>
       </c>
       <c r="D23">
-        <v>4</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PMXB43UNE</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C547273</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="E23" t="s">
+        <v>87</v>
+      </c>
+      <c r="F23" t="s">
+        <v>128</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -2803,27 +2796,25 @@
         </is>
       </c>
       <c r="H23">
-        <v>0.5428</v>
+        <v>0.0014</v>
       </c>
       <c r="I23" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>2.1712</v>
+        <v>0.0028</v>
+      </c>
+      <c r="J23">
+        <v>2930</v>
       </c>
       <c r="K23">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L23">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>124</v>
-      </c>
-      <c r="M23">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>124</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">New: deploy low-side FETs (Topology A); PMXB43UNEZ, unit cost is LCSC 100+ price (Oct 2026)</t>
-        </is>
+        <v>70</v>
+      </c>
+      <c r="M23" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.45">
@@ -2831,19 +2822,21 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
         <v>7</v>
       </c>
       <c r="D24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>87</v>
-      </c>
-      <c r="F24" t="s">
-        <v>128</v>
+        <v>175</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C25207446</t>
+        </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2851,33 +2844,33 @@
         </is>
       </c>
       <c r="H24">
-        <v>0.0014</v>
+        <v>0.0203</v>
       </c>
       <c r="I24" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0028</v>
+        <v>0.0203</v>
       </c>
       <c r="J24">
-        <v>2930</v>
+        <v>100</v>
       </c>
       <c r="K24">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L24">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="M24" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="C25" t="s">
         <v>7</v>
@@ -2885,122 +2878,122 @@
       <c r="D25">
         <v>1</v>
       </c>
-      <c r="E25" t="s">
-        <v>175</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C25207446</t>
-        </is>
+      <c r="E25">
+        <v>33</v>
+      </c>
+      <c r="F25" t="s">
+        <v>129</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H25">
-        <v>0.0203</v>
+        <v>0.0011</v>
       </c>
       <c r="I25" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0203</v>
+        <v>0.0011</v>
       </c>
       <c r="J25">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="K25">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L25">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="M25" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schematic value 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>49</v>
+        <v>183</v>
       </c>
       <c r="C26" t="s">
         <v>7</v>
       </c>
       <c r="D26">
-        <v>1</v>
-      </c>
-      <c r="E26">
-        <v>33</v>
+        <v>5</v>
+      </c>
+      <c r="E26" t="s">
+        <v>12</v>
       </c>
       <c r="F26" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H26">
-        <v>0.0011</v>
+        <v>0.0019</v>
       </c>
       <c r="I26" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0011</v>
+        <v>0.0095</v>
       </c>
       <c r="J26">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="K26">
         <v>10</v>
       </c>
       <c r="L26">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>40</v>
-      </c>
-      <c r="M26" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Schematic value 35</t>
-        </is>
+        <v>160</v>
+      </c>
+      <c r="M26">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" t="s">
-        <v>183</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R3,R17,R30</t>
+        </is>
       </c>
       <c r="C27" t="s">
         <v>7</v>
       </c>
       <c r="D27">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E27" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F27" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H27">
-        <v>0.0019</v>
+        <v>0.0015</v>
       </c>
       <c r="I27" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0095</v>
+        <v>0.0045</v>
       </c>
       <c r="J27">
         <v>150</v>
@@ -3010,33 +3003,31 @@
       </c>
       <c r="L27">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>160</v>
-      </c>
-      <c r="M27">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>10</v>
+        <v>100</v>
+      </c>
+      <c r="M27" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R3,R17,R30</t>
-        </is>
+      <c r="B28" t="s">
+        <v>96</v>
       </c>
       <c r="C28" t="s">
         <v>7</v>
       </c>
       <c r="D28">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E28" t="s">
-        <v>21</v>
+        <v>97</v>
       </c>
       <c r="F28" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -3044,21 +3035,21 @@
         </is>
       </c>
       <c r="H28">
-        <v>0.0015</v>
+        <v>0.0012</v>
       </c>
       <c r="I28" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0045</v>
+        <v>0.0012</v>
       </c>
       <c r="J28">
-        <v>150</v>
+        <v>74</v>
       </c>
       <c r="K28">
         <v>10</v>
       </c>
       <c r="L28">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="M28" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -3070,19 +3061,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>96</v>
+        <v>185</v>
       </c>
       <c r="C29" t="s">
         <v>7</v>
       </c>
       <c r="D29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" t="s">
-        <v>97</v>
+        <v>23</v>
       </c>
       <c r="F29" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -3090,21 +3081,21 @@
         </is>
       </c>
       <c r="H29">
-        <v>0.0012</v>
+        <v>0.0034</v>
       </c>
       <c r="I29" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0012</v>
+        <v>0.0068</v>
       </c>
       <c r="J29">
-        <v>74</v>
+        <v>890</v>
       </c>
       <c r="K29">
         <v>10</v>
       </c>
       <c r="L29">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="M29" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -3116,19 +3107,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C30" t="s">
         <v>7</v>
       </c>
       <c r="D30">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E30" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F30" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -3136,21 +3127,21 @@
         </is>
       </c>
       <c r="H30">
-        <v>0.0034</v>
+        <v>0.002</v>
       </c>
       <c r="I30" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0068</v>
+        <v>0.008</v>
       </c>
       <c r="J30">
-        <v>890</v>
+        <v>150</v>
       </c>
       <c r="K30">
         <v>10</v>
       </c>
       <c r="L30">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="M30" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -3162,41 +3153,41 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C31" t="s">
         <v>7</v>
       </c>
       <c r="D31">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E31" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F31" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H31">
-        <v>0.002</v>
+        <v>0.0026</v>
       </c>
       <c r="I31" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.008</v>
+        <v>0.0182</v>
       </c>
       <c r="J31">
-        <v>150</v>
+        <v>9705</v>
       </c>
       <c r="K31">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L31">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>130</v>
+        <v>222</v>
       </c>
       <c r="M31" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -3208,65 +3199,67 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="C32" t="s">
         <v>7</v>
       </c>
       <c r="D32">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E32" t="s">
-        <v>20</v>
+        <v>161</v>
       </c>
       <c r="F32" t="s">
-        <v>136</v>
+        <v>162</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H32">
-        <v>0.0026</v>
+        <v>0.0021</v>
       </c>
       <c r="I32" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0182</v>
+        <v>0.0042</v>
       </c>
       <c r="J32">
-        <v>9705</v>
+        <v>970</v>
       </c>
       <c r="K32">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L32">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>222</v>
+        <v>70</v>
       </c>
       <c r="M32" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33" t="s">
-        <v>160</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R4,R16,R19,R35,R43,R45,R46,R47,R48</t>
+        </is>
       </c>
       <c r="C33" t="s">
         <v>7</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E33" t="s">
-        <v>161</v>
+        <v>11</v>
       </c>
       <c r="F33" t="s">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -3274,51 +3267,54 @@
         </is>
       </c>
       <c r="H33">
-        <v>0.0021</v>
+        <v>0.0012</v>
       </c>
       <c r="I33" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0042</v>
+        <v>0.0108</v>
       </c>
       <c r="J33">
-        <v>970</v>
+        <v>960</v>
       </c>
       <c r="K33">
         <v>10</v>
       </c>
       <c r="L33">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>70</v>
+        <v>280</v>
       </c>
       <c r="M33" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schematic values R16=109, R19=98; R45-R48 are deploy FET gate resistors</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R4,R16,R19,R35,R43,R45,R46,R47,R48</t>
-        </is>
+      <c r="B34" t="s">
+        <v>28</v>
       </c>
       <c r="C34" t="s">
         <v>7</v>
       </c>
       <c r="D34">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E34" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F34" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H34">
@@ -3326,72 +3322,72 @@
       </c>
       <c r="I34" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0108</v>
+        <v>0.0036</v>
       </c>
       <c r="J34">
-        <v>960</v>
+        <v>2940</v>
       </c>
       <c r="K34">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L34">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>280</v>
+        <v>102</v>
       </c>
       <c r="M34" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Schematic values R16=109, R19=98; R45-R48 are deploy FET gate resistors</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.45">
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C35" t="s">
         <v>7</v>
       </c>
       <c r="D35">
-        <v>3</v>
-      </c>
-      <c r="E35" t="s">
-        <v>29</v>
+        <v>1</v>
+      </c>
+      <c r="E35">
+        <v>220</v>
       </c>
       <c r="F35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H35">
-        <v>0.0012</v>
+        <v>0.0018</v>
       </c>
       <c r="I35" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0036</v>
+        <v>0.0018</v>
       </c>
       <c r="J35">
-        <v>2940</v>
+        <v>3030</v>
       </c>
       <c r="K35">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L35">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>102</v>
+        <v>40</v>
       </c>
       <c r="M35" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schematic value 218</t>
+        </is>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.45">
@@ -3399,7 +3395,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="C36" t="s">
         <v>7</v>
@@ -3408,25 +3404,25 @@
         <v>1</v>
       </c>
       <c r="E36">
-        <v>220</v>
+        <v>374</v>
       </c>
       <c r="F36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H36">
-        <v>0.0018</v>
+        <v>0.0006</v>
       </c>
       <c r="I36" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0018</v>
+        <v>0.0006</v>
       </c>
       <c r="J36">
-        <v>3030</v>
+        <v>60</v>
       </c>
       <c r="K36">
         <v>10</v>
@@ -3441,16 +3437,16 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Schematic value 218</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.45">
+          <t xml:space="preserve">Schematic value 375</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="C37" t="s">
         <v>7</v>
@@ -3458,11 +3454,11 @@
       <c r="D37">
         <v>1</v>
       </c>
-      <c r="E37">
-        <v>374</v>
+      <c r="E37" t="s">
+        <v>99</v>
       </c>
       <c r="F37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -3470,11 +3466,11 @@
         </is>
       </c>
       <c r="H37">
-        <v>0.0006</v>
+        <v>0.0023</v>
       </c>
       <c r="I37" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0006</v>
+        <v>0.0023</v>
       </c>
       <c r="J37">
         <v>60</v>
@@ -3489,11 +3485,6 @@
       <c r="M37" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Schematic value 375</t>
-        </is>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.45">
@@ -3501,7 +3492,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="C38" t="s">
         <v>7</v>
@@ -3510,10 +3501,10 @@
         <v>1</v>
       </c>
       <c r="E38" t="s">
-        <v>99</v>
+        <v>176</v>
       </c>
       <c r="F38" t="s">
-        <v>140</v>
+        <v>173</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -3521,14 +3512,14 @@
         </is>
       </c>
       <c r="H38">
-        <v>0.0023</v>
+        <v>0.0213</v>
       </c>
       <c r="I38" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0023</v>
+        <v>0.0213</v>
       </c>
       <c r="J38">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="K38">
         <v>10</v>
@@ -3542,50 +3533,57 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A39">
         <v>38</v>
       </c>
-      <c r="B39" t="s">
-        <v>77</v>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R20,R29,R42,R44,R49,R50,R51,R52</t>
+        </is>
       </c>
       <c r="C39" t="s">
         <v>7</v>
       </c>
       <c r="D39">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E39" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="F39" t="s">
-        <v>173</v>
+        <v>141</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H39">
-        <v>0.0213</v>
+        <v>0.0015</v>
       </c>
       <c r="I39" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0213</v>
+        <v>0.012</v>
       </c>
       <c r="J39">
-        <v>100</v>
+        <v>4960</v>
       </c>
       <c r="K39">
         <v>10</v>
       </c>
       <c r="L39">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>40</v>
+        <v>250</v>
       </c>
       <c r="M39" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R20 was 1M before Topology A; R49-R52 are deploy FET gate pulldowns</t>
+        </is>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.45">
@@ -3594,20 +3592,26 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">R20,R29,R42,R44,R49,R50,R51,R52</t>
-        </is>
-      </c>
-      <c r="C40" t="s">
-        <v>7</v>
+          <t xml:space="preserve">R53,R54,R55,R56</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R_0402_1005Metric</t>
+        </is>
       </c>
       <c r="D40">
-        <v>8</v>
-      </c>
-      <c r="E40" t="s">
-        <v>164</v>
-      </c>
-      <c r="F40" t="s">
-        <v>141</v>
+        <v>4</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1K</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C11702</t>
+        </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -3615,86 +3619,73 @@
         </is>
       </c>
       <c r="H40">
-        <v>0.0015</v>
+        <v>0.0013</v>
       </c>
       <c r="I40" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.012</v>
-      </c>
-      <c r="J40">
-        <v>4960</v>
+        <v>0.0052</v>
       </c>
       <c r="K40">
         <v>10</v>
       </c>
       <c r="L40">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>250</v>
-      </c>
-      <c r="M40" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
+        <v>130</v>
+      </c>
+      <c r="M40">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v>130</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t xml:space="preserve">R20 was 1M before Topology A; R49-R52 are deploy FET gate pulldowns</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.45">
+          <t xml:space="preserve">New: DEPLOY1+..4+ bleeders (Topology A); unit cost is LCSC 100+ price (Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A41">
         <v>40</v>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R53,R54,R55,R56</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R_0402_1005Metric</t>
-        </is>
+      <c r="B41" t="s">
+        <v>190</v>
+      </c>
+      <c r="C41" t="s">
+        <v>13</v>
       </c>
       <c r="D41">
-        <v>4</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1K</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C11702</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="E41" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" t="s">
+        <v>142</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H41">
-        <v>0.0013</v>
+        <v>0.5919</v>
       </c>
       <c r="I41" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0052</v>
+        <v>2.9595</v>
+      </c>
+      <c r="J41">
+        <v>120</v>
       </c>
       <c r="K41">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L41">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="M41">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>130</v>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">New: DEPLOY1+..4+ bleeders (Topology A); unit cost is LCSC 100+ price (Oct 2026)</t>
-        </is>
+        <v>30</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.45">
@@ -3702,19 +3693,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>190</v>
+        <v>93</v>
       </c>
       <c r="C42" t="s">
-        <v>13</v>
+        <v>94</v>
       </c>
       <c r="D42">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E42" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="F42" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -3722,45 +3713,47 @@
         </is>
       </c>
       <c r="H42">
-        <v>0.5919</v>
+        <v>0.3336</v>
       </c>
       <c r="I42" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>2.9595</v>
+        <v>0.3336</v>
       </c>
       <c r="J42">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="K42">
         <v>0</v>
       </c>
       <c r="L42">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>150</v>
-      </c>
-      <c r="M42">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="M42" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>93</v>
-      </c>
-      <c r="C43" t="s">
-        <v>94</v>
+        <v>100</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WQFN 14 3.00 mm × 2.50 mm</t>
+        </is>
       </c>
       <c r="D43">
         <v>1</v>
       </c>
       <c r="E43" t="s">
-        <v>95</v>
+        <v>156</v>
       </c>
       <c r="F43" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -3768,14 +3761,14 @@
         </is>
       </c>
       <c r="H43">
-        <v>0.3336</v>
+        <v>0.3679</v>
       </c>
       <c r="I43" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.3336</v>
+        <v>0.3679</v>
       </c>
       <c r="J43">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="K43">
         <v>0</v>
@@ -3788,27 +3781,28 @@
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-    </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="Q43" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>100</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WQFN 14 3.00 mm × 2.50 mm</t>
-        </is>
+        <v>78</v>
+      </c>
+      <c r="C44" t="s">
+        <v>79</v>
       </c>
       <c r="D44">
         <v>1</v>
       </c>
       <c r="E44" t="s">
-        <v>156</v>
+        <v>80</v>
       </c>
       <c r="F44" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -3816,14 +3810,14 @@
         </is>
       </c>
       <c r="H44">
-        <v>0.3679</v>
+        <v>0.7504</v>
       </c>
       <c r="I44" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.3679</v>
+        <v>0.7504</v>
       </c>
       <c r="J44">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K44">
         <v>0</v>
@@ -3832,32 +3826,32 @@
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
         <v>30</v>
       </c>
-      <c r="M44" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
-      </c>
-      <c r="Q44" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="M44">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v>30</v>
+      </c>
+      <c r="N44">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>78</v>
+        <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>79</v>
+        <v>5</v>
       </c>
       <c r="D45">
         <v>1</v>
       </c>
       <c r="E45" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="F45" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -3865,14 +3859,14 @@
         </is>
       </c>
       <c r="H45">
-        <v>0.7504</v>
+        <v>14.1006</v>
       </c>
       <c r="I45" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.7504</v>
+        <v>14.1006</v>
       </c>
       <c r="J45">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K45">
         <v>0</v>
@@ -3881,12 +3875,9 @@
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
         <v>30</v>
       </c>
-      <c r="M45">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>30</v>
-      </c>
-      <c r="N45">
-        <v>34</v>
+      <c r="M45" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.45">
@@ -3894,19 +3885,19 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="C46" t="s">
-        <v>5</v>
+        <v>58</v>
       </c>
       <c r="D46">
         <v>1</v>
       </c>
       <c r="E46" t="s">
-        <v>6</v>
+        <v>59</v>
       </c>
       <c r="F46" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -3914,11 +3905,11 @@
         </is>
       </c>
       <c r="H46">
-        <v>14.1006</v>
+        <v>5.467</v>
       </c>
       <c r="I46" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>14.1006</v>
+        <v>5.467</v>
       </c>
       <c r="J46">
         <v>30</v>
@@ -3940,19 +3931,19 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>57</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>58</v>
+        <v>91</v>
       </c>
       <c r="D47">
         <v>1</v>
       </c>
       <c r="E47" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="F47" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -3960,11 +3951,11 @@
         </is>
       </c>
       <c r="H47">
-        <v>5.467</v>
+        <v>2.0322</v>
       </c>
       <c r="I47" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>5.467</v>
+        <v>2.0322</v>
       </c>
       <c r="J47">
         <v>30</v>
@@ -3981,24 +3972,24 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="C48" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="D48">
         <v>1</v>
       </c>
       <c r="E48" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="F48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -4006,14 +3997,14 @@
         </is>
       </c>
       <c r="H48">
-        <v>2.0322</v>
+        <v>1.1346</v>
       </c>
       <c r="I48" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>2.0322</v>
+        <v>1.1346</v>
       </c>
       <c r="J48">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K48">
         <v>0</v>
@@ -4022,29 +4013,32 @@
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
         <v>30</v>
       </c>
-      <c r="M48" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="M48">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v>30</v>
+      </c>
+      <c r="N48">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="C49" t="s">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="D49">
         <v>1</v>
       </c>
       <c r="E49" t="s">
-        <v>82</v>
+        <v>48</v>
       </c>
       <c r="F49" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -4052,14 +4046,14 @@
         </is>
       </c>
       <c r="H49">
-        <v>1.1346</v>
+        <v>20.5582</v>
       </c>
       <c r="I49" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>1.1346</v>
+        <v>20.5582</v>
       </c>
       <c r="J49">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K49">
         <v>0</v>
@@ -4068,12 +4062,9 @@
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
         <v>30</v>
       </c>
-      <c r="M49">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>30</v>
-      </c>
-      <c r="N49">
-        <v>30</v>
+      <c r="M49" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.45">
@@ -4081,19 +4072,19 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="C50" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="D50">
         <v>1</v>
       </c>
       <c r="E50" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="F50" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -4101,14 +4092,14 @@
         </is>
       </c>
       <c r="H50">
-        <v>20.5582</v>
+        <v>0.2927</v>
       </c>
       <c r="I50" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>20.5582</v>
+        <v>0.2927</v>
       </c>
       <c r="J50">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K50">
         <v>0</v>
@@ -4127,19 +4118,19 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="C51" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D51">
         <v>1</v>
       </c>
       <c r="E51" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="F51" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -4147,14 +4138,14 @@
         </is>
       </c>
       <c r="H51">
-        <v>0.2927</v>
+        <v>0.4284</v>
       </c>
       <c r="I51" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.2927</v>
+        <v>0.4284</v>
       </c>
       <c r="J51">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K51">
         <v>0</v>
@@ -4173,19 +4164,19 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="C52" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="F52" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -4193,11 +4184,11 @@
         </is>
       </c>
       <c r="H52">
-        <v>0.4284</v>
+        <v>24.6878</v>
       </c>
       <c r="I52" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.4284</v>
+        <v>24.6878</v>
       </c>
       <c r="J52">
         <v>30</v>
@@ -4219,19 +4210,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="C53" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="D53">
         <v>1</v>
       </c>
       <c r="E53" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="F53" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -4239,14 +4230,14 @@
         </is>
       </c>
       <c r="H53">
-        <v>24.6878</v>
+        <v>0.1196</v>
       </c>
       <c r="I53" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>24.6878</v>
+        <v>0.1196</v>
       </c>
       <c r="J53">
-        <v>30</v>
+        <v>127</v>
       </c>
       <c r="K53">
         <v>0</v>
@@ -4256,52 +4247,6 @@
         <v>30</v>
       </c>
       <c r="M53" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A54">
-        <v>53</v>
-      </c>
-      <c r="B54" t="s">
-        <v>72</v>
-      </c>
-      <c r="C54" t="s">
-        <v>73</v>
-      </c>
-      <c r="D54">
-        <v>1</v>
-      </c>
-      <c r="E54" t="s">
-        <v>74</v>
-      </c>
-      <c r="F54" t="s">
-        <v>153</v>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="H54">
-        <v>0.1196</v>
-      </c>
-      <c r="I54" s="3">
-        <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.1196</v>
-      </c>
-      <c r="J54">
-        <v>127</v>
-      </c>
-      <c r="K54">
-        <v>0</v>
-      </c>
-      <c r="L54">
-        <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>30</v>
-      </c>
-      <c r="M54" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add MMC5983MA magnetometer on I2C2
U19 MMC5983MA (JLCPCB C404329) joins the GPS I2C bus at 0x30 with
SPI_CS tied to VDDIO for I2C mode. C38 1uF on VDD, C39 0.1uF on VDDIO,
C37 10uF on CAP for the SET/RESET pulse. INT and SPI_SDO left unconnected.
Footprint is KiCad's stock Package_LGA:LGA-16_3x3mm_P0.5mm, which matches
the datasheet land pattern. New Custom:MMC5983MA symbol. BOM updated.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FYY8Uv6gBjRSv3QTZNtnYK
</commit_message>
<xml_diff>
--- a/BOM/RocketLocatorBOM.xlsx
+++ b/BOM/RocketLocatorBOM.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Assumptions" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="1" hidden="1">'RocketLocator'!$A$1:$E$53</definedName>
+    <definedName name="ExternalData_1" localSheetId="1" hidden="1">'RocketLocator'!$A$1:$E$54</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="199">
   <si>
     <t>Id</t>
   </si>
@@ -546,7 +546,7 @@
     <t>100K</t>
   </si>
   <si>
-    <t>C32</t>
+    <t>C32,C37</t>
   </si>
   <si>
     <t>4.7uF</t>
@@ -624,13 +624,28 @@
     <t>U1,U6,U8,U9,U15</t>
   </si>
   <si>
-    <t>C2,C3,C4,C5,C11,C12,C13,C14,C18</t>
+    <t>C2,C3,C4,C5,C11,C12,C13,C14,C18,C38</t>
   </si>
   <si>
     <t>C1,C6,C8,C9,C10,C20,C36</t>
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>U19</t>
+  </si>
+  <si>
+    <t>LGA-16_3x3mm_P0.5mm</t>
+  </si>
+  <si>
+    <t>MMC5983MA</t>
+  </si>
+  <si>
+    <t>C404329</t>
+  </si>
+  <si>
+    <t>Added 2026-10-21: magnetometer on I2C2 (0x30)</t>
   </si>
 </sst>
 </file>
@@ -756,10 +771,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}" name="RocketLocator" displayName="RocketLocator" ref="A1:Q53" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:Q53" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P53">
-    <sortCondition ref="B2:B53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}" name="RocketLocator" displayName="RocketLocator" ref="A1:Q54" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:Q54" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P54">
+    <sortCondition ref="B2:B54"/>
   </sortState>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{0660759B-7B44-48B6-BB59-01895697A8CF}" uniqueName="1" name="Id" queryTableFieldId="1"/>
@@ -1107,7 +1122,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61E55C0D-EF73-420E-9FF2-D4B1756536CB}">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.3984375" bestFit="1" customWidth="1"/>
@@ -1192,7 +1207,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C1,C6,C7,C8,C9,C10,C20,C36</t>
+          <t>C1,C6,C7,C8,C9,C10,C20,C36,C39</t>
         </is>
       </c>
       <c r="C6" t="s">
@@ -1788,6 +1803,20 @@
       </c>
       <c r="D46" t="s">
         <v>153</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A47" t="s">
+        <v>196</v>
+      </c>
+      <c r="B47" t="s">
+        <v>194</v>
+      </c>
+      <c r="C47" t="s">
+        <v>195</v>
+      </c>
+      <c r="D47" t="s">
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -1797,7 +1826,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E42B2C4-1B89-42AA-B989-7F67271C8485}">
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:Q54"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="4.46484375" bestFit="1" customWidth="1"/>
@@ -1979,7 +2008,7 @@
         <v>15</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="s">
         <v>65</v>
@@ -1997,7 +2026,7 @@
       </c>
       <c r="I4" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0257</v>
+        <v>0.0514</v>
       </c>
       <c r="J4">
         <v>930</v>
@@ -2007,7 +2036,7 @@
       </c>
       <c r="L4">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="M4" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -2028,7 +2057,7 @@
         <v>15</v>
       </c>
       <c r="D5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E5" t="s">
         <v>16</v>
@@ -2046,7 +2075,7 @@
       </c>
       <c r="I5" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0675</v>
+        <v>0.075</v>
       </c>
       <c r="J5">
         <v>480</v>
@@ -2056,7 +2085,7 @@
       </c>
       <c r="L5">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>280</v>
+        <v>310</v>
       </c>
       <c r="M5" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -2072,14 +2101,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C1,C6,C7,C8,C9,C10,C20,C36</t>
+          <t>C1,C6,C7,C8,C9,C10,C20,C36,C39</t>
         </is>
       </c>
       <c r="C6" t="s">
         <v>15</v>
       </c>
       <c r="D6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E6" t="s">
         <v>27</v>
@@ -2097,7 +2126,7 @@
       </c>
       <c r="I6" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0385</v>
+        <v>0.0495</v>
       </c>
       <c r="J6">
         <v>300</v>
@@ -2107,7 +2136,7 @@
       </c>
       <c r="L6">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>220</v>
+        <v>280</v>
       </c>
       <c r="M6" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -4249,6 +4278,52 @@
       <c r="M53" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>194</v>
+      </c>
+      <c r="C54" t="s">
+        <v>195</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+      <c r="E54" t="s">
+        <v>196</v>
+      </c>
+      <c r="F54" t="s">
+        <v>197</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="H54">
+        <v>1.843</v>
+      </c>
+      <c r="I54" s="3">
+        <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
+        <v>1.843</v>
+      </c>
+      <c r="K54">
+        <v>0</v>
+      </c>
+      <c r="L54">
+        <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
+        <v>30</v>
+      </c>
+      <c r="M54" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
+      </c>
+      <c r="Q54" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Drop C39 VDDIO bypass cap to match MMC5983MA datasheet
The datasheet application circuit has only 1uF on VDD (C38) and 10uF on
CAP (C37); VDD and VDDIO share +3V3 here, so C38 covers both.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FYY8Uv6gBjRSv3QTZNtnYK
</commit_message>
<xml_diff>
--- a/BOM/RocketLocatorBOM.xlsx
+++ b/BOM/RocketLocatorBOM.xlsx
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C1,C6,C7,C8,C9,C10,C20,C36,C39</t>
+          <t>C1,C6,C7,C8,C9,C10,C20,C36</t>
         </is>
       </c>
       <c r="C6" t="s">
@@ -2101,14 +2101,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C1,C6,C7,C8,C9,C10,C20,C36,C39</t>
+          <t>C1,C6,C7,C8,C9,C10,C20,C36</t>
         </is>
       </c>
       <c r="C6" t="s">
         <v>15</v>
       </c>
       <c r="D6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E6" t="s">
         <v>27</v>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="I6" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0495</v>
+        <v>0.044</v>
       </c>
       <c r="J6">
         <v>300</v>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="L6">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="M6" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>

</xml_diff>

<commit_message>
Space J12 battery pins and drop J3
J3 ("Battery-") was a separate pad so the battery leads could be
soldered apart. Return current through it ran along the bottom edge
past the U19 magnetometer. Instead, J12 now uses a 1x06 outline with
pads at positions 1-3 and 6 only, so +BATT sits 7.6 mm from the nearest
GND pad and every battery return enters at the top edge.

- New footprint Custom:PinHeader_1x06_P2.54mm_Vertical_Pos4-5_Empty.
  Pad numbers and nets are unchanged (1 GND, 2 MSW, 3 GND, 4 +BATT).
  Pad 4 is moved to position 6.
- Remove J3 and its GND symbol from the schematic.
- BOM: J12 footprint updated, J3 row removed (table now A1:Q53).

The PCB is not updated in this commit; run Update PCB from Schematic.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FYY8Uv6gBjRSv3QTZNtnYK
</commit_message>
<xml_diff>
--- a/BOM/RocketLocatorBOM.xlsx
+++ b/BOM/RocketLocatorBOM.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Assumptions" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="1" hidden="1">'RocketLocator'!$A$1:$E$54</definedName>
+    <definedName name="ExternalData_1" localSheetId="1" hidden="1">'RocketLocator'!$A$1:$E$53</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="200">
   <si>
     <t>Id</t>
   </si>
@@ -646,6 +646,9 @@
   </si>
   <si>
     <t>Added 2026-10-21: magnetometer on I2C2 (0x30)</t>
+  </si>
+  <si>
+    <t>PinHeader_1x06_P2.54mm_Vertical_Pos4-5_Empty</t>
   </si>
 </sst>
 </file>
@@ -771,10 +774,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}" name="RocketLocator" displayName="RocketLocator" ref="A1:Q54" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:Q54" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P54">
-    <sortCondition ref="B2:B54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}" name="RocketLocator" displayName="RocketLocator" ref="A1:Q53" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:Q53" xr:uid="{4C7D4CDA-AFCF-44BD-8318-990371684043}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P53">
+    <sortCondition ref="B2:B53"/>
   </sortState>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{0660759B-7B44-48B6-BB59-01895697A8CF}" uniqueName="1" name="Id" queryTableFieldId="1"/>
@@ -1826,7 +1829,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E42B2C4-1B89-42AA-B989-7F67271C8485}">
-  <dimension ref="A1:Q54"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="4.46484375" bestFit="1" customWidth="1"/>
@@ -2423,7 +2426,7 @@
         <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>199</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -2484,16 +2487,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="F15" t="s">
         <v>123</v>
@@ -2516,27 +2519,40 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" t="s">
-        <v>31</v>
+        <v>39</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HRS_U.FL-R-SMT(01)</t>
+        </is>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="F16" t="s">
-        <v>123</v>
+        <v>125</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="H16">
+        <v>0.0417</v>
       </c>
       <c r="I16" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
+        <v>0.0417</v>
+      </c>
+      <c r="J16">
+        <v>279</v>
       </c>
       <c r="L16">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="M16" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -2548,40 +2564,27 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HRS_U.FL-R-SMT(01)</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="C17" t="s">
+        <v>25</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="F17" t="s">
-        <v>125</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="H17">
-        <v>0.0417</v>
+        <v>123</v>
       </c>
       <c r="I17" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0417</v>
-      </c>
-      <c r="J17">
-        <v>279</v>
+        <v>0</v>
       </c>
       <c r="L17">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="M17" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -2593,16 +2596,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="C18" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="F18" t="s">
         <v>123</v>
@@ -2625,27 +2628,41 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>163</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="D19">
         <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="F19" t="s">
-        <v>123</v>
+        <v>126</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="H19">
+        <v>0.0218</v>
       </c>
       <c r="I19" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
+        <v>0.0218</v>
+      </c>
+      <c r="J19">
+        <v>75</v>
+      </c>
+      <c r="K19">
+        <v>5</v>
       </c>
       <c r="L19">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="M19" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -2657,7 +2674,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>163</v>
+        <v>17</v>
       </c>
       <c r="C20" t="s">
         <v>18</v>
@@ -2666,10 +2683,10 @@
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F20" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -2677,45 +2694,53 @@
         </is>
       </c>
       <c r="H20">
-        <v>0.0218</v>
+        <v>0.0403</v>
       </c>
       <c r="I20" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0218</v>
+        <v>0.0403</v>
       </c>
       <c r="J20">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="K20">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L20">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M20" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21" t="s">
-        <v>18</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q4,Q5,Q6,Q7</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nexperia_DFN1010D-3_SOT1215</t>
+        </is>
       </c>
       <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21" t="s">
-        <v>19</v>
-      </c>
-      <c r="F21" t="s">
-        <v>127</v>
+        <v>4</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PMXB43UNE</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C547273</t>
+        </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -2723,53 +2748,47 @@
         </is>
       </c>
       <c r="H21">
-        <v>0.0403</v>
+        <v>0.5428</v>
       </c>
       <c r="I21" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0403</v>
-      </c>
-      <c r="J21">
-        <v>42</v>
+        <v>2.1712</v>
       </c>
       <c r="K21">
         <v>4</v>
       </c>
       <c r="L21">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>34</v>
-      </c>
-      <c r="M21" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.45">
+        <v>124</v>
+      </c>
+      <c r="M21">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v>124</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New: deploy low-side FETs (Topology A); PMXB43UNEZ, unit cost is LCSC 100+ price (Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Q4,Q5,Q6,Q7</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nexperia_DFN1010D-3_SOT1215</t>
-        </is>
+      <c r="B22" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" t="s">
+        <v>7</v>
       </c>
       <c r="D22">
-        <v>4</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PMXB43UNE</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C547273</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="E22" t="s">
+        <v>87</v>
+      </c>
+      <c r="F22" t="s">
+        <v>128</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -2777,27 +2796,25 @@
         </is>
       </c>
       <c r="H22">
-        <v>0.5428</v>
+        <v>0.0014</v>
       </c>
       <c r="I22" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>2.1712</v>
+        <v>0.0028</v>
+      </c>
+      <c r="J22">
+        <v>2930</v>
       </c>
       <c r="K22">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L22">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>124</v>
-      </c>
-      <c r="M22">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>124</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">New: deploy low-side FETs (Topology A); PMXB43UNEZ, unit cost is LCSC 100+ price (Oct 2026)</t>
-        </is>
+        <v>70</v>
+      </c>
+      <c r="M22" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.45">
@@ -2805,19 +2822,21 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
         <v>7</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>87</v>
-      </c>
-      <c r="F23" t="s">
-        <v>128</v>
+        <v>175</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C25207446</t>
+        </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -2825,33 +2844,33 @@
         </is>
       </c>
       <c r="H23">
-        <v>0.0014</v>
+        <v>0.0203</v>
       </c>
       <c r="I23" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0028</v>
+        <v>0.0203</v>
       </c>
       <c r="J23">
-        <v>2930</v>
+        <v>100</v>
       </c>
       <c r="K23">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L23">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="M23" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="C24" t="s">
         <v>7</v>
@@ -2859,122 +2878,122 @@
       <c r="D24">
         <v>1</v>
       </c>
-      <c r="E24" t="s">
-        <v>175</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C25207446</t>
-        </is>
+      <c r="E24">
+        <v>33</v>
+      </c>
+      <c r="F24" t="s">
+        <v>129</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H24">
-        <v>0.0203</v>
+        <v>0.0011</v>
       </c>
       <c r="I24" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0203</v>
+        <v>0.0011</v>
       </c>
       <c r="J24">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="K24">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L24">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="M24" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schematic value 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>183</v>
       </c>
       <c r="C25" t="s">
         <v>7</v>
       </c>
       <c r="D25">
-        <v>1</v>
-      </c>
-      <c r="E25">
-        <v>33</v>
+        <v>5</v>
+      </c>
+      <c r="E25" t="s">
+        <v>12</v>
       </c>
       <c r="F25" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H25">
-        <v>0.0011</v>
+        <v>0.0019</v>
       </c>
       <c r="I25" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0011</v>
+        <v>0.0095</v>
       </c>
       <c r="J25">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="K25">
         <v>10</v>
       </c>
       <c r="L25">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>40</v>
-      </c>
-      <c r="M25" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Schematic value 35</t>
-        </is>
+        <v>160</v>
+      </c>
+      <c r="M25">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26" t="s">
-        <v>183</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R3,R17,R30</t>
+        </is>
       </c>
       <c r="C26" t="s">
         <v>7</v>
       </c>
       <c r="D26">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E26" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F26" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H26">
-        <v>0.0019</v>
+        <v>0.0015</v>
       </c>
       <c r="I26" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0095</v>
+        <v>0.0045</v>
       </c>
       <c r="J26">
         <v>150</v>
@@ -2984,33 +3003,31 @@
       </c>
       <c r="L26">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>160</v>
-      </c>
-      <c r="M26">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>10</v>
+        <v>100</v>
+      </c>
+      <c r="M26" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R3,R17,R30</t>
-        </is>
+      <c r="B27" t="s">
+        <v>96</v>
       </c>
       <c r="C27" t="s">
         <v>7</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E27" t="s">
-        <v>21</v>
+        <v>97</v>
       </c>
       <c r="F27" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -3018,21 +3035,21 @@
         </is>
       </c>
       <c r="H27">
-        <v>0.0015</v>
+        <v>0.0012</v>
       </c>
       <c r="I27" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0045</v>
+        <v>0.0012</v>
       </c>
       <c r="J27">
-        <v>150</v>
+        <v>74</v>
       </c>
       <c r="K27">
         <v>10</v>
       </c>
       <c r="L27">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="M27" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -3044,19 +3061,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>96</v>
+        <v>185</v>
       </c>
       <c r="C28" t="s">
         <v>7</v>
       </c>
       <c r="D28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" t="s">
-        <v>97</v>
+        <v>23</v>
       </c>
       <c r="F28" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -3064,21 +3081,21 @@
         </is>
       </c>
       <c r="H28">
-        <v>0.0012</v>
+        <v>0.0034</v>
       </c>
       <c r="I28" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0012</v>
+        <v>0.0068</v>
       </c>
       <c r="J28">
-        <v>74</v>
+        <v>890</v>
       </c>
       <c r="K28">
         <v>10</v>
       </c>
       <c r="L28">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="M28" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -3090,19 +3107,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C29" t="s">
         <v>7</v>
       </c>
       <c r="D29">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E29" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F29" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -3110,21 +3127,21 @@
         </is>
       </c>
       <c r="H29">
-        <v>0.0034</v>
+        <v>0.002</v>
       </c>
       <c r="I29" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0068</v>
+        <v>0.008</v>
       </c>
       <c r="J29">
-        <v>890</v>
+        <v>150</v>
       </c>
       <c r="K29">
         <v>10</v>
       </c>
       <c r="L29">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="M29" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -3136,41 +3153,41 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C30" t="s">
         <v>7</v>
       </c>
       <c r="D30">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E30" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F30" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H30">
-        <v>0.002</v>
+        <v>0.0026</v>
       </c>
       <c r="I30" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.008</v>
+        <v>0.0182</v>
       </c>
       <c r="J30">
-        <v>150</v>
+        <v>9705</v>
       </c>
       <c r="K30">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L30">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>130</v>
+        <v>222</v>
       </c>
       <c r="M30" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
@@ -3182,65 +3199,67 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="C31" t="s">
         <v>7</v>
       </c>
       <c r="D31">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E31" t="s">
-        <v>20</v>
+        <v>161</v>
       </c>
       <c r="F31" t="s">
-        <v>136</v>
+        <v>162</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H31">
-        <v>0.0026</v>
+        <v>0.0021</v>
       </c>
       <c r="I31" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0182</v>
+        <v>0.0042</v>
       </c>
       <c r="J31">
-        <v>9705</v>
+        <v>970</v>
       </c>
       <c r="K31">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L31">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>222</v>
+        <v>70</v>
       </c>
       <c r="M31" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>31</v>
       </c>
-      <c r="B32" t="s">
-        <v>160</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R4,R16,R19,R35,R43,R45,R46,R47,R48</t>
+        </is>
       </c>
       <c r="C32" t="s">
         <v>7</v>
       </c>
       <c r="D32">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E32" t="s">
-        <v>161</v>
+        <v>11</v>
       </c>
       <c r="F32" t="s">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -3248,51 +3267,54 @@
         </is>
       </c>
       <c r="H32">
-        <v>0.0021</v>
+        <v>0.0012</v>
       </c>
       <c r="I32" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0042</v>
+        <v>0.0108</v>
       </c>
       <c r="J32">
-        <v>970</v>
+        <v>960</v>
       </c>
       <c r="K32">
         <v>10</v>
       </c>
       <c r="L32">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>70</v>
+        <v>280</v>
       </c>
       <c r="M32" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schematic values R16=109, R19=98; R45-R48 are deploy FET gate resistors</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R4,R16,R19,R35,R43,R45,R46,R47,R48</t>
-        </is>
+      <c r="B33" t="s">
+        <v>28</v>
       </c>
       <c r="C33" t="s">
         <v>7</v>
       </c>
       <c r="D33">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E33" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F33" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H33">
@@ -3300,72 +3322,72 @@
       </c>
       <c r="I33" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0108</v>
+        <v>0.0036</v>
       </c>
       <c r="J33">
-        <v>960</v>
+        <v>2940</v>
       </c>
       <c r="K33">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L33">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>280</v>
+        <v>102</v>
       </c>
       <c r="M33" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Schematic values R16=109, R19=98; R45-R48 are deploy FET gate resistors</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.45">
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C34" t="s">
         <v>7</v>
       </c>
       <c r="D34">
-        <v>3</v>
-      </c>
-      <c r="E34" t="s">
-        <v>29</v>
+        <v>1</v>
+      </c>
+      <c r="E34">
+        <v>220</v>
       </c>
       <c r="F34" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H34">
-        <v>0.0012</v>
+        <v>0.0018</v>
       </c>
       <c r="I34" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0036</v>
+        <v>0.0018</v>
       </c>
       <c r="J34">
-        <v>2940</v>
+        <v>3030</v>
       </c>
       <c r="K34">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L34">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>102</v>
+        <v>40</v>
       </c>
       <c r="M34" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schematic value 218</t>
+        </is>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.45">
@@ -3373,7 +3395,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="C35" t="s">
         <v>7</v>
@@ -3382,25 +3404,25 @@
         <v>1</v>
       </c>
       <c r="E35">
-        <v>220</v>
+        <v>374</v>
       </c>
       <c r="F35" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H35">
-        <v>0.0018</v>
+        <v>0.0006</v>
       </c>
       <c r="I35" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0018</v>
+        <v>0.0006</v>
       </c>
       <c r="J35">
-        <v>3030</v>
+        <v>60</v>
       </c>
       <c r="K35">
         <v>10</v>
@@ -3415,16 +3437,16 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Schematic value 218</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.45">
+          <t xml:space="preserve">Schematic value 375</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="C36" t="s">
         <v>7</v>
@@ -3432,11 +3454,11 @@
       <c r="D36">
         <v>1</v>
       </c>
-      <c r="E36">
-        <v>374</v>
+      <c r="E36" t="s">
+        <v>99</v>
       </c>
       <c r="F36" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -3444,11 +3466,11 @@
         </is>
       </c>
       <c r="H36">
-        <v>0.0006</v>
+        <v>0.0023</v>
       </c>
       <c r="I36" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0006</v>
+        <v>0.0023</v>
       </c>
       <c r="J36">
         <v>60</v>
@@ -3463,11 +3485,6 @@
       <c r="M36" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Schematic value 375</t>
-        </is>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.45">
@@ -3475,7 +3492,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="C37" t="s">
         <v>7</v>
@@ -3484,10 +3501,10 @@
         <v>1</v>
       </c>
       <c r="E37" t="s">
-        <v>99</v>
+        <v>176</v>
       </c>
       <c r="F37" t="s">
-        <v>140</v>
+        <v>173</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -3495,14 +3512,14 @@
         </is>
       </c>
       <c r="H37">
-        <v>0.0023</v>
+        <v>0.0213</v>
       </c>
       <c r="I37" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0023</v>
+        <v>0.0213</v>
       </c>
       <c r="J37">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="K37">
         <v>10</v>
@@ -3516,50 +3533,57 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>37</v>
       </c>
-      <c r="B38" t="s">
-        <v>77</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R20,R29,R42,R44,R49,R50,R51,R52</t>
+        </is>
       </c>
       <c r="C38" t="s">
         <v>7</v>
       </c>
       <c r="D38">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E38" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="F38" t="s">
-        <v>173</v>
+        <v>141</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H38">
-        <v>0.0213</v>
+        <v>0.0015</v>
       </c>
       <c r="I38" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0213</v>
+        <v>0.012</v>
       </c>
       <c r="J38">
-        <v>100</v>
+        <v>4960</v>
       </c>
       <c r="K38">
         <v>10</v>
       </c>
       <c r="L38">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>40</v>
+        <v>250</v>
       </c>
       <c r="M38" t="str">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R20 was 1M before Topology A; R49-R52 are deploy FET gate pulldowns</t>
+        </is>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.45">
@@ -3568,20 +3592,26 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">R20,R29,R42,R44,R49,R50,R51,R52</t>
-        </is>
-      </c>
-      <c r="C39" t="s">
-        <v>7</v>
+          <t xml:space="preserve">R53,R54,R55,R56</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R_0402_1005Metric</t>
+        </is>
       </c>
       <c r="D39">
-        <v>8</v>
-      </c>
-      <c r="E39" t="s">
-        <v>164</v>
-      </c>
-      <c r="F39" t="s">
-        <v>141</v>
+        <v>4</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1K</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C11702</t>
+        </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -3589,86 +3619,73 @@
         </is>
       </c>
       <c r="H39">
-        <v>0.0015</v>
+        <v>0.0013</v>
       </c>
       <c r="I39" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.012</v>
-      </c>
-      <c r="J39">
-        <v>4960</v>
+        <v>0.0052</v>
       </c>
       <c r="K39">
         <v>10</v>
       </c>
       <c r="L39">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>250</v>
-      </c>
-      <c r="M39" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
+        <v>130</v>
+      </c>
+      <c r="M39">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v>130</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t xml:space="preserve">R20 was 1M before Topology A; R49-R52 are deploy FET gate pulldowns</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.45">
+          <t xml:space="preserve">New: DEPLOY1+..4+ bleeders (Topology A); unit cost is LCSC 100+ price (Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A40">
         <v>39</v>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R53,R54,R55,R56</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R_0402_1005Metric</t>
-        </is>
+      <c r="B40" t="s">
+        <v>190</v>
+      </c>
+      <c r="C40" t="s">
+        <v>13</v>
       </c>
       <c r="D40">
-        <v>4</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1K</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C11702</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>142</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="H40">
-        <v>0.0013</v>
+        <v>0.5919</v>
       </c>
       <c r="I40" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.0052</v>
+        <v>2.9595</v>
+      </c>
+      <c r="J40">
+        <v>120</v>
       </c>
       <c r="K40">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L40">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="M40">
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>130</v>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">New: DEPLOY1+..4+ bleeders (Topology A); unit cost is LCSC 100+ price (Oct 2026)</t>
-        </is>
+        <v>30</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.45">
@@ -3676,19 +3693,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>190</v>
+        <v>93</v>
       </c>
       <c r="C41" t="s">
-        <v>13</v>
+        <v>94</v>
       </c>
       <c r="D41">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E41" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="F41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -3696,45 +3713,47 @@
         </is>
       </c>
       <c r="H41">
-        <v>0.5919</v>
+        <v>0.3336</v>
       </c>
       <c r="I41" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>2.9595</v>
+        <v>0.3336</v>
       </c>
       <c r="J41">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="K41">
         <v>0</v>
       </c>
       <c r="L41">
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>150</v>
-      </c>
-      <c r="M41">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="M41" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>93</v>
-      </c>
-      <c r="C42" t="s">
-        <v>94</v>
+        <v>100</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WQFN 14 3.00 mm × 2.50 mm</t>
+        </is>
       </c>
       <c r="D42">
         <v>1</v>
       </c>
       <c r="E42" t="s">
-        <v>95</v>
+        <v>156</v>
       </c>
       <c r="F42" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -3742,14 +3761,14 @@
         </is>
       </c>
       <c r="H42">
-        <v>0.3336</v>
+        <v>0.3679</v>
       </c>
       <c r="I42" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.3336</v>
+        <v>0.3679</v>
       </c>
       <c r="J42">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="K42">
         <v>0</v>
@@ -3762,27 +3781,28 @@
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-    </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="Q42" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>100</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WQFN 14 3.00 mm × 2.50 mm</t>
-        </is>
+        <v>78</v>
+      </c>
+      <c r="C43" t="s">
+        <v>79</v>
       </c>
       <c r="D43">
         <v>1</v>
       </c>
       <c r="E43" t="s">
-        <v>156</v>
+        <v>80</v>
       </c>
       <c r="F43" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -3790,14 +3810,14 @@
         </is>
       </c>
       <c r="H43">
-        <v>0.3679</v>
+        <v>0.7504</v>
       </c>
       <c r="I43" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.3679</v>
+        <v>0.7504</v>
       </c>
       <c r="J43">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K43">
         <v>0</v>
@@ -3806,32 +3826,32 @@
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
         <v>30</v>
       </c>
-      <c r="M43" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
-      </c>
-      <c r="Q43" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="M43">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v>30</v>
+      </c>
+      <c r="N43">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>78</v>
+        <v>4</v>
       </c>
       <c r="C44" t="s">
-        <v>79</v>
+        <v>5</v>
       </c>
       <c r="D44">
         <v>1</v>
       </c>
       <c r="E44" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="F44" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -3839,14 +3859,14 @@
         </is>
       </c>
       <c r="H44">
-        <v>0.7504</v>
+        <v>14.1006</v>
       </c>
       <c r="I44" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.7504</v>
+        <v>14.1006</v>
       </c>
       <c r="J44">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K44">
         <v>0</v>
@@ -3855,12 +3875,9 @@
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
         <v>30</v>
       </c>
-      <c r="M44">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>30</v>
-      </c>
-      <c r="N44">
-        <v>34</v>
+      <c r="M44" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.45">
@@ -3868,19 +3885,19 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="C45" t="s">
-        <v>5</v>
+        <v>58</v>
       </c>
       <c r="D45">
         <v>1</v>
       </c>
       <c r="E45" t="s">
-        <v>6</v>
+        <v>59</v>
       </c>
       <c r="F45" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -3888,11 +3905,11 @@
         </is>
       </c>
       <c r="H45">
-        <v>14.1006</v>
+        <v>5.467</v>
       </c>
       <c r="I45" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>14.1006</v>
+        <v>5.467</v>
       </c>
       <c r="J45">
         <v>30</v>
@@ -3914,19 +3931,19 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>57</v>
+        <v>90</v>
       </c>
       <c r="C46" t="s">
-        <v>58</v>
+        <v>91</v>
       </c>
       <c r="D46">
         <v>1</v>
       </c>
       <c r="E46" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="F46" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -3934,11 +3951,11 @@
         </is>
       </c>
       <c r="H46">
-        <v>5.467</v>
+        <v>2.0322</v>
       </c>
       <c r="I46" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>5.467</v>
+        <v>2.0322</v>
       </c>
       <c r="J46">
         <v>30</v>
@@ -3955,24 +3972,24 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="C47" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="D47">
         <v>1</v>
       </c>
       <c r="E47" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="F47" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -3980,14 +3997,14 @@
         </is>
       </c>
       <c r="H47">
-        <v>2.0322</v>
+        <v>1.1346</v>
       </c>
       <c r="I47" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>2.0322</v>
+        <v>1.1346</v>
       </c>
       <c r="J47">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K47">
         <v>0</v>
@@ -3996,29 +4013,32 @@
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
         <v>30</v>
       </c>
-      <c r="M47" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="M47">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v>30</v>
+      </c>
+      <c r="N47">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="C48" t="s">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="D48">
         <v>1</v>
       </c>
       <c r="E48" t="s">
-        <v>82</v>
+        <v>48</v>
       </c>
       <c r="F48" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -4026,14 +4046,14 @@
         </is>
       </c>
       <c r="H48">
-        <v>1.1346</v>
+        <v>20.5582</v>
       </c>
       <c r="I48" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>1.1346</v>
+        <v>20.5582</v>
       </c>
       <c r="J48">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K48">
         <v>0</v>
@@ -4042,12 +4062,9 @@
         <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
         <v>30</v>
       </c>
-      <c r="M48">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v>30</v>
-      </c>
-      <c r="N48">
-        <v>30</v>
+      <c r="M48" t="str">
+        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
+        <v/>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.45">
@@ -4055,19 +4072,19 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="C49" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="D49">
         <v>1</v>
       </c>
       <c r="E49" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="F49" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -4075,14 +4092,14 @@
         </is>
       </c>
       <c r="H49">
-        <v>20.5582</v>
+        <v>0.2927</v>
       </c>
       <c r="I49" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>20.5582</v>
+        <v>0.2927</v>
       </c>
       <c r="J49">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K49">
         <v>0</v>
@@ -4101,19 +4118,19 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="C50" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D50">
         <v>1</v>
       </c>
       <c r="E50" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="F50" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -4121,14 +4138,14 @@
         </is>
       </c>
       <c r="H50">
-        <v>0.2927</v>
+        <v>0.4284</v>
       </c>
       <c r="I50" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.2927</v>
+        <v>0.4284</v>
       </c>
       <c r="J50">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K50">
         <v>0</v>
@@ -4147,19 +4164,19 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="C51" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="D51">
         <v>1</v>
       </c>
       <c r="E51" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="F51" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -4167,11 +4184,11 @@
         </is>
       </c>
       <c r="H51">
-        <v>0.4284</v>
+        <v>24.6878</v>
       </c>
       <c r="I51" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.4284</v>
+        <v>24.6878</v>
       </c>
       <c r="J51">
         <v>30</v>
@@ -4193,19 +4210,19 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="C52" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="F52" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -4213,14 +4230,14 @@
         </is>
       </c>
       <c r="H52">
-        <v>24.6878</v>
+        <v>0.1196</v>
       </c>
       <c r="I52" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>24.6878</v>
+        <v>0.1196</v>
       </c>
       <c r="J52">
-        <v>30</v>
+        <v>127</v>
       </c>
       <c r="K52">
         <v>0</v>
@@ -4234,24 +4251,24 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>72</v>
+        <v>194</v>
       </c>
       <c r="C53" t="s">
-        <v>73</v>
+        <v>195</v>
       </c>
       <c r="D53">
         <v>1</v>
       </c>
       <c r="E53" t="s">
-        <v>74</v>
+        <v>196</v>
       </c>
       <c r="F53" t="s">
-        <v>153</v>
+        <v>197</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -4259,14 +4276,11 @@
         </is>
       </c>
       <c r="H53">
-        <v>0.1196</v>
+        <v>1.843</v>
       </c>
       <c r="I53" s="3">
         <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>0.1196</v>
-      </c>
-      <c r="J53">
-        <v>127</v>
+        <v>1.843</v>
       </c>
       <c r="K53">
         <v>0</v>
@@ -4279,50 +4293,7 @@
         <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
         <v/>
       </c>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.45">
-      <c r="A54">
-        <v>53</v>
-      </c>
-      <c r="B54" t="s">
-        <v>194</v>
-      </c>
-      <c r="C54" t="s">
-        <v>195</v>
-      </c>
-      <c r="D54">
-        <v>1</v>
-      </c>
-      <c r="E54" t="s">
-        <v>196</v>
-      </c>
-      <c r="F54" t="s">
-        <v>197</v>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="H54">
-        <v>1.843</v>
-      </c>
-      <c r="I54" s="3">
-        <f>RocketLocator[[#This Row],[Quantity]]*RocketLocator[[#This Row],[Unit Cost]]</f>
-        <v>1.843</v>
-      </c>
-      <c r="K54">
-        <v>0</v>
-      </c>
-      <c r="L54">
-        <f>IF(AND(RocketLocator[[#This Row],[Quantity]]&gt;0,RocketLocator[[#This Row],[JLCPCB Part '#（optional）]]&lt;&gt;"N/A"),Assumptions!$B$1*RocketLocator[[#This Row],[Quantity]]+RocketLocator[[#This Row],[Attrition Quantity]],0)</f>
-        <v>30</v>
-      </c>
-      <c r="M54" t="str">
-        <f>IF(RocketLocator[[#This Row],[Quantity Needed]]&gt;RocketLocator[[#This Row],[Quantity on Hand]],RocketLocator[[#This Row],[Quantity Needed]]-RocketLocator[[#This Row],[Quantity on Hand]],"")</f>
-        <v/>
-      </c>
-      <c r="Q54" t="s">
+      <c r="Q53" t="s">
         <v>198</v>
       </c>
     </row>

</xml_diff>